<commit_message>
feat: add behavior guidelines to conversation agent persona
</commit_message>
<xml_diff>
--- a/prompt_tone_tracker.xlsx
+++ b/prompt_tone_tracker.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">

</xml_diff>